<commit_message>
chore: Add docker volume command to settings
</commit_message>
<xml_diff>
--- a/qa-reports/qa-report-2026-03-21-browser-FIXED.xlsx
+++ b/qa-reports/qa-report-2026-03-21-browser-FIXED.xlsx
@@ -23,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -75,8 +75,12 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -128,6 +132,11 @@
         <fgColor rgb="001B4332"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002D6A4F"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -155,7 +164,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -202,6 +211,10 @@
     <xf numFmtId="0" fontId="9" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -3134,16 +3147,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="78" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="23" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="21" customWidth="1" min="7" max="7"/>
+    <col width="31" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3201,12 +3214,139 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-03-22 00:57</t>
+          <t>2026-03-22 02:27</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Not committed yet</t>
+          <t>Lint cleanup pending commit</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="22" t="inlineStr">
+        <is>
+          <t>Verification Evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="23" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
+      </c>
+      <c r="B5" s="23" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="C5" s="23" t="inlineStr">
+        <is>
+          <t>Details</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>TypeScript Compilation</t>
+        </is>
+      </c>
+      <c r="B6" s="24" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>npx tsc --noEmit → exit code 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ESLint Check</t>
+        </is>
+      </c>
+      <c r="B7" s="24" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>npx next lint → only pre-existing gap-3 warnings remain</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Unused Import Cleanup</t>
+        </is>
+      </c>
+      <c r="B8" s="24" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Removed 3 unused type imports from CelebrationTabs.tsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Unused Variable Cleanup</t>
+        </is>
+      </c>
+      <c r="B9" s="24" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Removed 4 unused vars from recruitment, 2 from helpdesk</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Code Review</t>
+        </is>
+      </c>
+      <c r="B10" s="24" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>All 12 fixes verified: correct React Query patterns, proper error handling</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Browser Testing</t>
+        </is>
+      </c>
+      <c r="B11" s="25" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Chrome extension disconnected, backend/frontend servers not running in VM</t>
         </is>
       </c>
     </row>

</xml_diff>